<commit_message>
Đồng bộ mã nguồn chuẩn từ máy tính
</commit_message>
<xml_diff>
--- a/tailieu/SO_TAY_KTV.xlsx
+++ b/tailieu/SO_TAY_KTV.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="27">
   <si>
     <t>Triển khai dịch vụ Internet</t>
   </si>
@@ -159,12 +159,6 @@
   </si>
   <si>
     <t>Bán hàng</t>
-  </si>
-  <si>
-    <t>hello</t>
-  </si>
-  <si>
-    <t>iohaiohhho</t>
   </si>
 </sst>
 </file>
@@ -660,15 +654,7 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>27</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C13" t="s">
-        <v>20</v>
-      </c>
+      <c r="B13" s="1"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="B14" s="1"/>

</xml_diff>